<commit_message>
Streaming control test - Command test
</commit_message>
<xml_diff>
--- a/doc/K2CoverageResults.xlsx
+++ b/doc/K2CoverageResults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\openSUSE-Tumbleweed\home\ssilvestri\research\Kappa2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D1BD6A-78B6-47B1-B898-5F419B1BAA83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FD9A299-9209-46D3-A7C2-6C7449CB23E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{834EB836-E108-4946-BBD2-E48878051BC8}"/>
   </bookViews>
@@ -18,7 +18,6 @@
     <sheet name="KCoder" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -349,19 +348,19 @@
                   <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>35</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>36</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>64</c:v>
+                  <c:v>67</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -456,19 +455,19 @@
                   <c:v>91</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>230</c:v>
+                  <c:v>244</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>205</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>239</c:v>
+                  <c:v>243</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>51</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>444</c:v>
+                  <c:v>522</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -563,19 +562,19 @@
                   <c:v>247</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>466</c:v>
+                  <c:v>495</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>393</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>530</c:v>
+                  <c:v>549</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>80</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1189</c:v>
+                  <c:v>1367</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -901,28 +900,28 @@
                   <c:v>94.855305466237937</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>60</c:v>
+                  <c:v>53.333333333333336</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>79.365079365079367</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>98.785425101214571</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>81.330472103004297</c:v>
+                  <c:v>86.868686868686879</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>94.402035623409674</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>89.433962264150949</c:v>
+                  <c:v>86.338797814207652</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>78.132884777123635</c:v>
+                  <c:v>86.027798098024874</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1218,10 +1217,10 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>82.521405373486871</c:v>
+                  <c:v>88.292277885413782</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17.478594626513129</c:v>
+                  <c:v>11.707722114586218</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5428,24 +5427,24 @@
         <v>33.333333333333329</v>
       </c>
       <c r="E3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F3">
         <v>20</v>
       </c>
       <c r="G3" s="1">
         <f t="shared" ref="G3:G12" si="1">E3/F3*100</f>
-        <v>55.000000000000007</v>
+        <v>50</v>
       </c>
       <c r="H3">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I3">
         <v>45</v>
       </c>
       <c r="J3" s="1">
         <f t="shared" ref="J3:J12" si="2">H3/I3*100</f>
-        <v>60</v>
+        <v>53.333333333333336</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -5473,14 +5472,14 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I4">
         <v>126</v>
       </c>
       <c r="J4" s="1">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>79.365079365079367</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -5523,34 +5522,34 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C6">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="0"/>
-        <v>65.714285714285708</v>
+        <v>65.853658536585371</v>
       </c>
       <c r="E6">
-        <v>186</v>
+        <v>215</v>
       </c>
       <c r="F6">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="G6" s="1">
         <f t="shared" si="1"/>
-        <v>80.869565217391298</v>
+        <v>88.114754098360663</v>
       </c>
       <c r="H6">
-        <v>379</v>
+        <v>430</v>
       </c>
       <c r="I6">
-        <v>466</v>
+        <v>495</v>
       </c>
       <c r="J6" s="1">
         <f t="shared" si="2"/>
-        <v>81.330472103004297</v>
+        <v>86.868686868686879</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -5596,31 +5595,31 @@
         <v>32</v>
       </c>
       <c r="C8">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1">
         <f t="shared" si="0"/>
-        <v>88.888888888888886</v>
+        <v>86.486486486486484</v>
       </c>
       <c r="E8">
         <v>223</v>
       </c>
       <c r="F8">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="G8" s="1">
         <f t="shared" si="1"/>
-        <v>93.305439330543933</v>
+        <v>91.769547325102891</v>
       </c>
       <c r="H8">
         <v>474</v>
       </c>
       <c r="I8">
-        <v>530</v>
+        <v>549</v>
       </c>
       <c r="J8" s="1">
         <f t="shared" si="2"/>
-        <v>89.433962264150949</v>
+        <v>86.338797814207652</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -5663,34 +5662,34 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C10">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D10" s="1">
         <f t="shared" si="0"/>
-        <v>46.875</v>
+        <v>59.701492537313428</v>
       </c>
       <c r="E10">
-        <v>346</v>
+        <v>449</v>
       </c>
       <c r="F10">
-        <v>444</v>
+        <v>522</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" si="1"/>
-        <v>77.927927927927925</v>
+        <v>86.015325670498086</v>
       </c>
       <c r="H10">
-        <v>929</v>
+        <v>1176</v>
       </c>
       <c r="I10">
-        <v>1189</v>
+        <v>1367</v>
       </c>
       <c r="J10" s="1">
         <f t="shared" si="2"/>
-        <v>78.132884777123635</v>
+        <v>86.027798098024874</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -5699,39 +5698,39 @@
       </c>
       <c r="B12">
         <f>SUM(B2:B10)</f>
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C12">
         <f t="shared" ref="C12:I12" si="3">SUM(C2:C10)</f>
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="D12" s="1">
         <f t="shared" si="0"/>
-        <v>67.307692307692307</v>
+        <v>70.642201834862391</v>
       </c>
       <c r="E12">
         <f t="shared" si="3"/>
-        <v>1215</v>
+        <v>1346</v>
       </c>
       <c r="F12">
         <f t="shared" si="3"/>
-        <v>1483</v>
+        <v>1579</v>
       </c>
       <c r="G12" s="1">
         <f t="shared" si="1"/>
-        <v>81.928523263654753</v>
+        <v>85.243825205826468</v>
       </c>
       <c r="H12">
         <f t="shared" si="3"/>
-        <v>2795</v>
+        <v>3190</v>
       </c>
       <c r="I12">
         <f t="shared" si="3"/>
-        <v>3387</v>
+        <v>3613</v>
       </c>
       <c r="J12" s="1">
         <f t="shared" si="2"/>
-        <v>82.521405373486871</v>
+        <v>88.292277885413782</v>
       </c>
       <c r="K12" t="s">
         <v>23</v>
@@ -5740,7 +5739,7 @@
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="J13" s="1">
         <f>100-J12</f>
-        <v>17.478594626513129</v>
+        <v>11.707722114586218</v>
       </c>
       <c r="K13" t="s">
         <v>24</v>
@@ -5752,7 +5751,7 @@
       </c>
       <c r="M18">
         <f>I12-I4</f>
-        <v>3261</v>
+        <v>3487</v>
       </c>
     </row>
     <row r="19" spans="12:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Test for Syntax Tree finish
</commit_message>
<xml_diff>
--- a/doc/K2CoverageResults.xlsx
+++ b/doc/K2CoverageResults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\openSUSE-Tumbleweed\home\ssilvestri\research\Kappa2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44993DEE-DCA9-4B0A-8661-0CFF074E3D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6A63A8-D3C2-4368-9919-F35FF5DE7894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{834EB836-E108-4946-BBD2-E48878051BC8}"/>
   </bookViews>
@@ -97,9 +97,6 @@
     <t>Phase 2</t>
   </si>
   <si>
-    <t>ast.rs</t>
-  </si>
-  <si>
     <t>coder.rs</t>
   </si>
   <si>
@@ -113,6 +110,9 @@
   </si>
   <si>
     <t>Uncovered</t>
+  </si>
+  <si>
+    <t>syntax_tree.rs</t>
   </si>
 </sst>
 </file>
@@ -1411,6 +1411,9 @@
         <c:ser>
           <c:idx val="1"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>Functions</c:v>
+          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:schemeClr val="accent2"/>
@@ -1427,13 +1430,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>ast.rs</c:v>
+                  <c:v>coder.rs</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>coder.rs</c:v>
+                  <c:v>parser.rs</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>parser.rs</c:v>
+                  <c:v>syntax_tree.rs</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1445,13 +1448,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>31</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>23</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>27</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1465,6 +1468,9 @@
         <c:ser>
           <c:idx val="4"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>Lines</c:v>
+          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:schemeClr val="accent5"/>
@@ -1481,13 +1487,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>ast.rs</c:v>
+                  <c:v>coder.rs</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>coder.rs</c:v>
+                  <c:v>parser.rs</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>parser.rs</c:v>
+                  <c:v>syntax_tree.rs</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1499,13 +1505,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>430</c:v>
+                  <c:v>329</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>329</c:v>
+                  <c:v>325</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>325</c:v>
+                  <c:v>526</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1519,6 +1525,9 @@
         <c:ser>
           <c:idx val="7"/>
           <c:order val="2"/>
+          <c:tx>
+            <c:v>Regions</c:v>
+          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:schemeClr val="accent2">
@@ -1537,13 +1546,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>ast.rs</c:v>
+                  <c:v>coder.rs</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>coder.rs</c:v>
+                  <c:v>parser.rs</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>parser.rs</c:v>
+                  <c:v>syntax_tree.rs</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1555,13 +1564,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>847</c:v>
+                  <c:v>621</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>621</c:v>
+                  <c:v>592</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>592</c:v>
+                  <c:v>1169</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1898,13 +1907,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>ast.rs</c:v>
+                  <c:v>coder.rs</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>coder.rs</c:v>
+                  <c:v>parser.rs</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>parser.rs</c:v>
+                  <c:v>syntax_tree.rs</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1916,13 +1925,13 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.23612750885478156</c:v>
+                  <c:v>0.322061191626409</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.322061191626409</c:v>
+                  <c:v>89.86486486486487</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>89.86486486486487</c:v>
+                  <c:v>86.4841745081266</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2055,7 +2064,7 @@
       </c:valAx>
       <c:spPr>
         <a:noFill/>
-        <a:ln>
+        <a:ln w="25400">
           <a:noFill/>
         </a:ln>
         <a:effectLst/>
@@ -5733,7 +5742,7 @@
         <v>88.292277885413782</v>
       </c>
       <c r="K12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -5742,7 +5751,7 @@
         <v>11.707722114586218</v>
       </c>
       <c r="K13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="12:13" x14ac:dyDescent="0.3">
@@ -5773,6 +5782,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B342025-DC6A-446C-A7CB-D53CF62D5F59}">
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
@@ -5808,31 +5820,31 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D2" s="1">
-        <f>B2/C2*100</f>
-        <v>3.225806451612903</v>
+        <f t="shared" ref="D2:D3" si="0">B2/C2*100</f>
+        <v>4.3478260869565215</v>
       </c>
       <c r="E2">
         <v>2</v>
       </c>
       <c r="F2">
-        <v>430</v>
+        <v>329</v>
       </c>
       <c r="G2" s="1">
-        <f>E2/F2*100</f>
-        <v>0.46511627906976744</v>
+        <f t="shared" ref="G2:G3" si="1">E2/F2*100</f>
+        <v>0.60790273556231</v>
       </c>
       <c r="H2">
         <v>2</v>
       </c>
       <c r="I2">
-        <v>847</v>
+        <v>621</v>
       </c>
       <c r="J2" s="1">
-        <f>H2/I2*100</f>
-        <v>0.23612750885478156</v>
+        <f t="shared" ref="J2:J3" si="2">H2/I2*100</f>
+        <v>0.322061191626409</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -5840,69 +5852,69 @@
         <v>20</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C3">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D3" s="1">
-        <f t="shared" ref="D3:D4" si="0">B3/C3*100</f>
-        <v>4.3478260869565215</v>
+        <f t="shared" si="0"/>
+        <v>77.777777777777786</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>290</v>
       </c>
       <c r="F3">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="G3" s="1">
-        <f t="shared" ref="G3:G4" si="1">E3/F3*100</f>
-        <v>0.60790273556231</v>
+        <f t="shared" si="1"/>
+        <v>89.230769230769241</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>532</v>
       </c>
       <c r="I3">
-        <v>621</v>
+        <v>592</v>
       </c>
       <c r="J3" s="1">
-        <f t="shared" ref="J3:J4" si="2">H3/I3*100</f>
-        <v>0.322061191626409</v>
+        <f t="shared" si="2"/>
+        <v>89.86486486486487</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B4">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C4">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="D4" s="1">
-        <f t="shared" si="0"/>
-        <v>77.777777777777786</v>
+        <f>B4/C4*100</f>
+        <v>81.081081081081081</v>
       </c>
       <c r="E4">
-        <v>290</v>
+        <v>437</v>
       </c>
       <c r="F4">
-        <v>325</v>
+        <v>526</v>
       </c>
       <c r="G4" s="1">
-        <f t="shared" si="1"/>
-        <v>89.230769230769241</v>
+        <f>E4/F4*100</f>
+        <v>83.079847908745251</v>
       </c>
       <c r="H4">
-        <v>532</v>
+        <v>1011</v>
       </c>
       <c r="I4">
-        <v>592</v>
+        <v>1169</v>
       </c>
       <c r="J4" s="1">
-        <f t="shared" si="2"/>
-        <v>89.86486486486487</v>
+        <f>H4/I4*100</f>
+        <v>86.4841745081266</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -5910,40 +5922,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <f>SUM(B2:B4)</f>
-        <v>23</v>
+        <f>SUM(B2:B3)</f>
+        <v>22</v>
       </c>
       <c r="C6">
-        <f>SUM(C2:C4)</f>
-        <v>81</v>
+        <f>SUM(C2:C3)</f>
+        <v>50</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" ref="D6" si="3">B6/C6*100</f>
-        <v>28.39506172839506</v>
+        <v>44</v>
       </c>
       <c r="E6">
-        <f>SUM(E2:E4)</f>
-        <v>294</v>
+        <f>SUM(E2:E3)</f>
+        <v>292</v>
       </c>
       <c r="F6">
-        <f>SUM(F2:F4)</f>
-        <v>1084</v>
+        <f>SUM(F2:F3)</f>
+        <v>654</v>
       </c>
       <c r="G6" s="1">
         <f t="shared" ref="G6" si="4">E6/F6*100</f>
-        <v>27.121771217712176</v>
+        <v>44.648318042813457</v>
       </c>
       <c r="H6">
-        <f>SUM(H2:H4)</f>
-        <v>536</v>
+        <f>SUM(H2:H3)</f>
+        <v>534</v>
       </c>
       <c r="I6">
-        <f>SUM(I2:I4)</f>
-        <v>2060</v>
+        <f>SUM(I2:I3)</f>
+        <v>1213</v>
       </c>
       <c r="J6" s="1">
         <f t="shared" ref="J6" si="5">H6/I6*100</f>
-        <v>26.019417475728158</v>
+        <v>44.023083264633136</v>
       </c>
     </row>
   </sheetData>
@@ -5985,7 +5997,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2">
         <v>0</v>

</xml_diff>